<commit_message>
BSI.IT.27.C7.05: add 'Evidence Needed to Pass' tab
Lists what blocks a pass, a 12-item evidence request list with provider and
pass criteria, a per-account checklist for the 16 accounts / 30 memberships
in exceptions E1-E3, and how the result will be re-assessed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GtAt3iBzX5VYFEMTgXwPkP
</commit_message>
<xml_diff>
--- a/BSI.IT.27.C7 Network Device Admin Accoun/BSI.IT.27.C7.05 Testing Walkthrough - Step by Step.xlsx
+++ b/BSI.IT.27.C7 Network Device Admin Accoun/BSI.IT.27.C7.05 Testing Walkthrough - Step by Step.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4_Item Detail (58)" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5_Exceptions E1-E3" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6_Sources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7_Evidence Needed to Pass" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4_Item Detail (58)'!$A$3:$W$61</definedName>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -64,8 +65,14 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF9C0006"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -97,6 +104,11 @@
         <fgColor rgb="FFFFC000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -124,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -158,6 +170,13 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10209,6 +10228,7 @@
         </is>
       </c>
     </row>
+    <row r="36"/>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="11" t="inlineStr">
         <is>
@@ -10623,4 +10643,1617 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Additional evidence required to clear the exceptions and pending items - BSI.IT.27.C7 (2026 Q2 sample)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="62" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>IMPORTANT: the result can change to PASS only if the evidence shows the access was appropriate at the time of the review (e.g. the identity was active with a valid, extended contract and the IAMS flag / termination date was wrong, or the re-grant followed an approved access request). If the evidence confirms the users were inactive / terminated or the re-grant was not approved, the exception stands: removing the access now is remediation (tracked as an issue / action driver) and does not change the result of this sample - the control would be re-tested in the next cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>1. What is preventing a PASS today</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Attr.</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Why it is not Pass</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Items affected</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>What changes it to Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Appropriateness of approved access</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Approved privileged network access for identities inactive (E1) / terminated (E2) in IAMS and for memberships re-granted after 2025 Q3 revocation (E3).</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>30 memberships (CISCO Network Administrators 16, ISEAdmin 14)</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Evidence per account (section 3) proving each approval was appropriate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Frequency (at least semiannual)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>No certification evidenced between 2025 Q3 (Aug 2025) and 2026 Q2 (Jul 2026).</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Control period</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>2025 Q4 and/or 2026 Q1 certification reports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>PENDING (partial)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Completeness vs Active Directory</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Current AD membership of the 4 groups not provided; completeness only corroborated to the CyberArk certification.</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>4 groups</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>AD extract reconciled to the certified members (differences explained).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>PASS (gap)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Decision dates</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>SOX Manager export ("Validation1") has no Decision Date / SignOff Date.</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>48 person memberships</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Standard SailPoint decision report with dates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>OBSERVATION</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Information reliability</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Account Status "Account Removed" on all owner / CyberArk records; Manager export lacks status fields.</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Reports</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Explanation of the field + report parameters (IPE).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>2. Evidence request list (send to control owner / PAM team)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Attribute</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Evidence to request</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>What the evidence must show to PASS</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>If not provided / not as expected</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Received (Y/N)</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Date received</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>A5 - E1</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>HR / vendor contract status of the 5 consultants flagged Identity Inactive in IAMS (X688027, X689040, X689379, X690623, X690995) as of the review date (8/17/2026).</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>HR / Vendor management; IAM team</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>HR record or signed contract / SOW showing active engagement on 7/22-8/17/2026, and IAMS explanation of why Identity Inactive = True.</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>Access remains an exception (approved for inactive identities).</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="n"/>
+      <c r="I14" s="13" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>A5 - E1</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Active Directory account detail for the same 5 accounts: enabled flag, accountExpires, lastLogonDate, memberOf (Cisco Network Administrators, ISEAdmin, Network_support).</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>BSI IT Operations (AD extract, same script as 2025 Cycle 2)</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Accounts enabled and used consistently with an active engagement; or disabled / removed before the review close.</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Confirms inappropriate access; request removal evidence (Netwrix) for remediation.</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="n"/>
+      <c r="I15" s="13" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>A5 - E2</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>HR record / contract extension for the 8 identities with IAMS Termination Date 12/31/2024 (MIA25103, MIA25104, MIA25105, MIA25106, MIA25142, MIA25249, MIA25250, MIA25251).</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>HR / Vendor management; IAM team</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Contract extended beyond 12/31/2024 and still active at the review date; IAMS termination date shown to be an outdated data field (with ticket correcting it).</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Access remains an exception (approved for terminated identities in 2025 Q3 and 2026 Q2).</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="n"/>
+      <c r="I16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>A5 - E2</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>AD account detail (enabled, lastLogonDate, accountExpires) for the 8 MIA252xx accounts.</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>BSI IT Operations</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Accounts active and legitimately used after 12/31/2024.</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>Confirms exception.</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="n"/>
+      <c r="I17" s="13" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>A5 - E3</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Access request and approvals for the re-grant of X453396, MIA25142 (Cisco Network Administrators and ISEAdmin), MIA25172 and MIA25175 (Cisco Network Administrators) after the 2025 Q3 revocation.</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>PAM / IAM team (ServiceNow / SailPoint request)</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Request identifying the group, approved by the user's manager and the group owner / S-CISO BEFORE the membership was added; business justification.</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Re-grant without approval - exception stands.</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="n"/>
+      <c r="I18" s="13" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>A5 - E3</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Netwrix / AD change log showing who added the 6 memberships back and when (after 9/2-9/8/2025 removal).</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>BSI InfoSec (Netwrix Auditor)</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Add date after the approval date in item 5; performed by authorized PAM/IAM personnel.</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Provisioning before approval - exception stands.</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="n"/>
+      <c r="I19" s="13" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>A5 - all</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Reviewer (Dayam Borges) explanation / supporting analysis for approving the E1-E3 memberships on 8/17/2026.</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>Control owner</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>Documented, reasonable basis for each approval (e.g. contract verified).</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Supports conclusion that review precision is insufficient.</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="n"/>
+      <c r="I20" s="13" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>2025 Q4 and 2026 Q1 PAM BSI SOX Manager and Entitlement Owner certification decision reports (or evidence the campaigns were launched), OR management confirmation they were not performed.</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>IAM / PAM team (SailPoint)</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>At least one certification of the 4 groups launched between 8/2025 and 2/2026 so no gap exceeds 6 months.</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Frequency exception (gap ~12 months &gt; semiannual).</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" s="13" t="n"/>
+      <c r="I21" s="13" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Current AD membership extract of CISCO ISE Administrators, CISCO Network Administrators, ISEAdmin and F5FullAdmin (dated, with the script used).</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>BSI IT Operations</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>All current members were certified in 2026 Q2 or added after the campaign with an approved request (Netwrix add log).</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Completeness exception for uncertified members.</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="n"/>
+      <c r="I22" s="13" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>A4 / A7</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>SailPoint 2026 Q2 SOX Manager Certification standard decision report (Decision Date, SignOff Date, Identity Inactive, Termination Date) + screenshot of the campaign status (Completed).</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>IAM / PAM team</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Decisions and sign-off within the campaign period; fields consistent with the Validation1 export.</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Decision timing not evidenced (observation).</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="n"/>
+      <c r="I23" s="13" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Explanation of the "Account Status = Account Removed" field in the Daily Active exports and the report parameters / run date.</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>IAM team</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Field meaning understood; report complete and accurate (IPE).</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Observation remains.</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="n"/>
+      <c r="I24" s="13" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>A2 (scope)</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Management confirmation whether mia.usa.sinvest\Network_support ("Network devices Administrators", PAM Definition sec. 3.2) is in scope of BSI.IT.27.C7.</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>InfoSec / control owner</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Documented scope decision; if in scope, the same evidence (items 1-4) also covers its 5 inactive members.</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Scope observation.</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H25" s="13" t="n"/>
+      <c r="I25" s="13" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>3. Per-account checklist - A5 exceptions (fill "Received" and "Re-test result" when evidence arrives)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Group(s)</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>Exception</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Evidence needed</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>Pass condition</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>Memberships</t>
+        </is>
+      </c>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>Received (Y/N)</t>
+        </is>
+      </c>
+      <c r="J28" s="9" t="inlineStr">
+        <is>
+          <t>Re-test result</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>MIA25103</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Ramirez Gonzalez, Ivan</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Contract extension beyond 12/31/2024 + AD detail (req. 3-4)</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Contract extended and active at the review date; termination date outdated</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I29" s="14" t="inlineStr"/>
+      <c r="J29" s="14" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>MIA25104</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Paez Venegas, Jefferson</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Contract extension beyond 12/31/2024 + AD detail (req. 3-4)</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Contract extended and active at the review date; termination date outdated</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I30" s="14" t="inlineStr"/>
+      <c r="J30" s="14" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>MIA25105</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Serrano Aguirre, David</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Contract extension beyond 12/31/2024 + AD detail (req. 3-4)</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>Contract extended and active at the review date; termination date outdated</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I31" s="14" t="inlineStr"/>
+      <c r="J31" s="14" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>MIA25106</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Vazquez Arias, Maiko</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Contract extension beyond 12/31/2024 + AD detail (req. 3-4)</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Contract extended and active at the review date; termination date outdated</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I32" s="14" t="inlineStr"/>
+      <c r="J32" s="14" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>MIA25142</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Nieves Nieves, Miguel</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>E2, E3</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Contract extension beyond 12/31/2024 + AD detail (req. 3-4)
+Approved access request (manager + group owner / S-CISO) + Netwrix add log for the re-grant (req. 5-6)</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Contract extended and active at the review date; termination date outdated
+Re-grant approved before provisioning by manager and group owner</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I33" s="14" t="inlineStr"/>
+      <c r="J33" s="14" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>MIA25172</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Hernandez Ruiz, Juan</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Approved access request (manager + group owner / S-CISO) + Netwrix add log for the re-grant (req. 5-6)</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Re-grant approved before provisioning by manager and group owner</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" s="14" t="inlineStr"/>
+      <c r="J34" s="14" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>MIA25175</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Hernandez Acevedo, Carlos</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Approved access request (manager + group owner / S-CISO) + Netwrix add log for the re-grant (req. 5-6)</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Re-grant approved before provisioning by manager and group owner</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I35" s="14" t="inlineStr"/>
+      <c r="J35" s="14" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>MIA25249</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Harris, Richard</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>Contract extension beyond 12/31/2024 + AD detail (req. 3-4)</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>Contract extended and active at the review date; termination date outdated</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I36" s="14" t="inlineStr"/>
+      <c r="J36" s="14" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>MIA25250</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Ackley, Kevin</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>Contract extension beyond 12/31/2024 + AD detail (req. 3-4)</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>Contract extended and active at the review date; termination date outdated</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I37" s="14" t="inlineStr"/>
+      <c r="J37" s="14" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>MIA25251</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Rimal, Ashish</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Contract extension beyond 12/31/2024 + AD detail (req. 3-4)</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>Contract extended and active at the review date; termination date outdated</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I38" s="14" t="inlineStr"/>
+      <c r="J38" s="14" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>X453396</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Perez Peralta, Juan Fernando</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>Approved access request (manager + group owner / S-CISO) + Netwrix add log for the re-grant (req. 5-6)</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Re-grant approved before provisioning by manager and group owner</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I39" s="14" t="inlineStr"/>
+      <c r="J39" s="14" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>X688027</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Guzman, Yazir</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>HR / contract status at 8/17/2026 + AD enabled / lastLogon (req. 1-2)</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>Identity active and engagement valid at the review date; IAMS flag incorrect</t>
+        </is>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I40" s="14" t="inlineStr"/>
+      <c r="J40" s="14" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>X689040</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>Vazquez Hernandez, Jesus</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>HR / contract status at 8/17/2026 + AD enabled / lastLogon (req. 1-2)</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>Identity active and engagement valid at the review date; IAMS flag incorrect</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I41" s="14" t="inlineStr"/>
+      <c r="J41" s="14" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>X689379</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Martinez Cervantes, Pamela</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>HR / contract status at 8/17/2026 + AD enabled / lastLogon (req. 1-2)</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>Identity active and engagement valid at the review date; IAMS flag incorrect</t>
+        </is>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I42" s="14" t="inlineStr"/>
+      <c r="J42" s="14" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>X690623</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Jimenez, Carlos</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>HR / contract status at 8/17/2026 + AD enabled / lastLogon (req. 1-2)</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>Identity active and engagement valid at the review date; IAMS flag incorrect</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I43" s="14" t="inlineStr"/>
+      <c r="J43" s="14" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>X690995</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Martinez, Jose Antonio</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>CISCO Network Administrators; ISEAdmin</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>HR / contract status at 8/17/2026 + AD enabled / lastLogon (req. 1-2)</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>Identity active and engagement valid at the review date; IAMS flag incorrect</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I44" s="14" t="inlineStr"/>
+      <c r="J44" s="14" t="inlineStr"/>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>Total: 16 accounts / 30 memberships to clear. All must be cleared (and A1 evidenced) for the 2026 Q2 sample to PASS; any account not cleared keeps CISCO Network Administrators / ISEAdmin as FAIL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>4. How the result will be re-assessed</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="32" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Evidence outcome</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Result for A5 / sample</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Next action</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>All E1-E3 accounts supported</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Contracts valid, IAMS flags wrong (with correction ticket); re-grants approved before provisioning</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>A5 PASS</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Record IAMS data-quality observation; confirm A1 evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Some accounts supported</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Only part of the 16 accounts supported</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>A5 FAIL for the remaining accounts</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>Exception stands; raise issue for the unsupported accounts</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Users inactive / terminated confirmed</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>HR confirms end of engagement; access still active at review</t>
+        </is>
+      </c>
+      <c r="D52" s="8" t="inlineStr">
+        <is>
+          <t>A5 FAIL</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Issue / action driver: remove access (Netwrix evidence), root cause of review precision</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Re-grant without approval</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>No request or approval after provisioning date</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>A5 FAIL</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>Issue: provisioning outside process; remove or formally approve</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>A1 frequency</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>2025 Q4 / 2026 Q1 certification provided</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>A1 PASS</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Otherwise A1 FAIL - frequency deficiency (gap &gt; 6 months)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A46:J46"/>
+    <mergeCell ref="A27:J27"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A4:J4"/>
+    <mergeCell ref="A48:J48"/>
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>